<commit_message>
Improve full notification downloads, pagination, retries, and localhost paging
</commit_message>
<xml_diff>
--- a/downloads/Notificaciones Electrónicas.xlsx
+++ b/downloads/Notificaciones Electrónicas.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="78">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="93">
   <si>
     <t>Nro. Notificación</t>
   </si>
@@ -44,33 +44,81 @@
     <t>Estado de lectura</t>
   </si>
   <si>
+    <t>202600040663-4</t>
+  </si>
+  <si>
+    <t>RUC 20103117560</t>
+  </si>
+  <si>
+    <t>EMP REG DE SERV PUB DE ELECT DL NORTE SA</t>
+  </si>
+  <si>
+    <t/>
+  </si>
+  <si>
+    <t>202600040663</t>
+  </si>
+  <si>
+    <t>Trámite Electrónico</t>
+  </si>
+  <si>
+    <t>Declarar la aplicación del silencio administrativo positivo.</t>
+  </si>
+  <si>
+    <t>16/03/2026 02:00:59 PM</t>
+  </si>
+  <si>
+    <t>No leída</t>
+  </si>
+  <si>
+    <t>202600039598-4</t>
+  </si>
+  <si>
+    <t>202600039598</t>
+  </si>
+  <si>
+    <t>16/03/2026 01:37:16 PM</t>
+  </si>
+  <si>
+    <t>202600036344-2</t>
+  </si>
+  <si>
+    <t>202600036344</t>
+  </si>
+  <si>
+    <t>EN RPTA A RESOLUCIÓN JARU N° 1226-2026-OS/JARU-S2, APELACION DE GALVEZ CUEVA DORIS MADELEINE, EXP. N° 202600005656, RES. 25100094811, REC. R93787-C-2025, SUM. 25810305.</t>
+  </si>
+  <si>
+    <t>16/03/2026 01:33:29 PM</t>
+  </si>
+  <si>
+    <t>202600042210-2</t>
+  </si>
+  <si>
+    <t>202600042210</t>
+  </si>
+  <si>
+    <t>QUEJA POR SAP: SUM. 26844424 (EXC. FACTURA AGOSTO 25, STIEMBRE 25, OCTUBRE 25 Y NOVIEMBRE 25)</t>
+  </si>
+  <si>
+    <t>16/03/2026 01:32:13 PM</t>
+  </si>
+  <si>
+    <t>Leída</t>
+  </si>
+  <si>
     <t>202500114631-4</t>
   </si>
   <si>
-    <t>RUC 20103117560</t>
-  </si>
-  <si>
-    <t>EMP REG DE SERV PUB DE ELECT DL NORTE SA</t>
-  </si>
-  <si>
-    <t/>
-  </si>
-  <si>
     <t>202500114631</t>
   </si>
   <si>
-    <t>Trámite Electrónico</t>
-  </si>
-  <si>
     <t>Brochure_CalidadSuministro_2025T1</t>
   </si>
   <si>
     <t>16/03/2026 12:45:57 PM</t>
   </si>
   <si>
-    <t>No leída</t>
-  </si>
-  <si>
     <t>202500300443-2</t>
   </si>
   <si>
@@ -93,9 +141,6 @@
   </si>
   <si>
     <t>16/03/2026 12:35:03 PM</t>
-  </si>
-  <si>
-    <t>Leída</t>
   </si>
   <si>
     <t>202600048979-2</t>
@@ -385,10 +430,10 @@
         <v>15</v>
       </c>
       <c r="H3" t="s" s="1">
+        <v>16</v>
+      </c>
+      <c r="I3" t="s" s="1">
         <v>21</v>
-      </c>
-      <c r="I3" t="s" s="1">
-        <v>22</v>
       </c>
       <c r="K3" t="s" s="1">
         <v>18</v>
@@ -396,418 +441,546 @@
     </row>
     <row r="4">
       <c r="A4" t="s" s="1">
+        <v>22</v>
+      </c>
+      <c r="B4" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="C4" t="s" s="1">
+        <v>12</v>
+      </c>
+      <c r="D4" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E4" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="F4" t="s" s="1">
         <v>23</v>
       </c>
-      <c r="B4" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="C4" t="s" s="1">
-        <v>12</v>
-      </c>
-      <c r="D4" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E4" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="F4" t="s" s="1">
+      <c r="G4" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="H4" t="s" s="1">
         <v>24</v>
       </c>
-      <c r="G4" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="H4" t="s" s="1">
+      <c r="I4" t="s" s="1">
         <v>25</v>
       </c>
-      <c r="I4" t="s" s="1">
-        <v>26</v>
-      </c>
       <c r="K4" t="s" s="1">
-        <v>27</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="1">
+        <v>26</v>
+      </c>
+      <c r="B5" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s" s="1">
+        <v>12</v>
+      </c>
+      <c r="D5" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E5" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="F5" t="s" s="1">
+        <v>27</v>
+      </c>
+      <c r="G5" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="H5" t="s" s="1">
         <v>28</v>
       </c>
-      <c r="B5" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="C5" t="s" s="1">
-        <v>12</v>
-      </c>
-      <c r="D5" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E5" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="F5" t="s" s="1">
+      <c r="I5" t="s" s="1">
         <v>29</v>
       </c>
-      <c r="G5" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="H5" t="s" s="1">
-        <v>30</v>
-      </c>
-      <c r="I5" t="s" s="1">
-        <v>31</v>
-      </c>
       <c r="K5" t="s" s="1">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="1">
+        <v>31</v>
+      </c>
+      <c r="B6" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="C6" t="s" s="1">
+        <v>12</v>
+      </c>
+      <c r="D6" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E6" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="F6" t="s" s="1">
         <v>32</v>
       </c>
-      <c r="B6" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="C6" t="s" s="1">
-        <v>12</v>
-      </c>
-      <c r="D6" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E6" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="F6" t="s" s="1">
+      <c r="G6" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="H6" t="s" s="1">
         <v>33</v>
       </c>
-      <c r="G6" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="H6" t="s" s="1">
+      <c r="I6" t="s" s="1">
         <v>34</v>
       </c>
-      <c r="I6" t="s" s="1">
-        <v>35</v>
-      </c>
       <c r="K6" t="s" s="1">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="1">
+        <v>35</v>
+      </c>
+      <c r="B7" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="C7" t="s" s="1">
+        <v>12</v>
+      </c>
+      <c r="D7" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E7" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="F7" t="s" s="1">
         <v>36</v>
       </c>
-      <c r="B7" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="C7" t="s" s="1">
-        <v>12</v>
-      </c>
-      <c r="D7" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E7" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="F7" t="s" s="1">
+      <c r="G7" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="H7" t="s" s="1">
         <v>37</v>
       </c>
-      <c r="G7" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="H7" t="s" s="1">
+      <c r="I7" t="s" s="1">
         <v>38</v>
       </c>
-      <c r="I7" t="s" s="1">
-        <v>39</v>
-      </c>
       <c r="K7" t="s" s="1">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="1">
+        <v>39</v>
+      </c>
+      <c r="B8" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="C8" t="s" s="1">
+        <v>12</v>
+      </c>
+      <c r="D8" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E8" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="F8" t="s" s="1">
         <v>40</v>
       </c>
-      <c r="B8" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="C8" t="s" s="1">
-        <v>12</v>
-      </c>
-      <c r="D8" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E8" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="F8" t="s" s="1">
+      <c r="G8" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="H8" t="s" s="1">
         <v>41</v>
       </c>
-      <c r="G8" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="H8" t="s" s="1">
+      <c r="I8" t="s" s="1">
         <v>42</v>
       </c>
-      <c r="I8" t="s" s="1">
-        <v>43</v>
-      </c>
       <c r="K8" t="s" s="1">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="1">
+        <v>43</v>
+      </c>
+      <c r="B9" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="C9" t="s" s="1">
+        <v>12</v>
+      </c>
+      <c r="D9" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E9" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="F9" t="s" s="1">
         <v>44</v>
       </c>
-      <c r="B9" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="C9" t="s" s="1">
-        <v>12</v>
-      </c>
-      <c r="D9" t="s" s="1">
+      <c r="G9" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="H9" t="s" s="1">
         <v>45</v>
       </c>
-      <c r="E9" t="s" s="1">
+      <c r="I9" t="s" s="1">
         <v>46</v>
       </c>
-      <c r="F9" t="s" s="1">
-        <v>47</v>
-      </c>
-      <c r="G9" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="H9" t="s" s="1">
-        <v>48</v>
-      </c>
-      <c r="I9" t="s" s="1">
-        <v>49</v>
-      </c>
       <c r="K9" t="s" s="1">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="1">
+        <v>47</v>
+      </c>
+      <c r="B10" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="C10" t="s" s="1">
+        <v>12</v>
+      </c>
+      <c r="D10" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E10" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="F10" t="s" s="1">
+        <v>48</v>
+      </c>
+      <c r="G10" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="H10" t="s" s="1">
+        <v>49</v>
+      </c>
+      <c r="I10" t="s" s="1">
         <v>50</v>
       </c>
-      <c r="B10" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="C10" t="s" s="1">
-        <v>12</v>
-      </c>
-      <c r="D10" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E10" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="F10" t="s" s="1">
-        <v>51</v>
-      </c>
-      <c r="G10" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="H10" t="s" s="1">
-        <v>52</v>
-      </c>
-      <c r="I10" t="s" s="1">
-        <v>53</v>
-      </c>
       <c r="K10" t="s" s="1">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="1">
+        <v>51</v>
+      </c>
+      <c r="B11" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="C11" t="s" s="1">
+        <v>12</v>
+      </c>
+      <c r="D11" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E11" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="F11" t="s" s="1">
+        <v>52</v>
+      </c>
+      <c r="G11" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="H11" t="s" s="1">
+        <v>53</v>
+      </c>
+      <c r="I11" t="s" s="1">
         <v>54</v>
       </c>
-      <c r="B11" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="C11" t="s" s="1">
-        <v>12</v>
-      </c>
-      <c r="D11" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E11" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="F11" t="s" s="1">
-        <v>55</v>
-      </c>
-      <c r="G11" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="H11" t="s" s="1">
-        <v>56</v>
-      </c>
-      <c r="I11" t="s" s="1">
-        <v>57</v>
-      </c>
       <c r="K11" t="s" s="1">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="1">
+        <v>55</v>
+      </c>
+      <c r="B12" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="C12" t="s" s="1">
+        <v>12</v>
+      </c>
+      <c r="D12" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E12" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="F12" t="s" s="1">
+        <v>56</v>
+      </c>
+      <c r="G12" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="H12" t="s" s="1">
+        <v>57</v>
+      </c>
+      <c r="I12" t="s" s="1">
         <v>58</v>
       </c>
-      <c r="B12" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="C12" t="s" s="1">
-        <v>12</v>
-      </c>
-      <c r="D12" t="s" s="1">
-        <v>45</v>
-      </c>
-      <c r="E12" t="s" s="1">
-        <v>46</v>
-      </c>
-      <c r="F12" t="s" s="1">
-        <v>59</v>
-      </c>
-      <c r="G12" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="H12" t="s" s="1">
-        <v>60</v>
-      </c>
-      <c r="I12" t="s" s="1">
-        <v>61</v>
-      </c>
       <c r="K12" t="s" s="1">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="1">
+        <v>59</v>
+      </c>
+      <c r="B13" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="C13" t="s" s="1">
+        <v>12</v>
+      </c>
+      <c r="D13" t="s" s="1">
+        <v>60</v>
+      </c>
+      <c r="E13" t="s" s="1">
+        <v>61</v>
+      </c>
+      <c r="F13" t="s" s="1">
         <v>62</v>
       </c>
-      <c r="B13" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="C13" t="s" s="1">
-        <v>12</v>
-      </c>
-      <c r="D13" t="s" s="1">
-        <v>45</v>
-      </c>
-      <c r="E13" t="s" s="1">
-        <v>46</v>
-      </c>
-      <c r="F13" t="s" s="1">
+      <c r="G13" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="H13" t="s" s="1">
         <v>63</v>
       </c>
-      <c r="G13" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="H13" t="s" s="1">
+      <c r="I13" t="s" s="1">
         <v>64</v>
       </c>
-      <c r="I13" t="s" s="1">
-        <v>65</v>
-      </c>
       <c r="K13" t="s" s="1">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="1">
+        <v>65</v>
+      </c>
+      <c r="B14" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="C14" t="s" s="1">
+        <v>12</v>
+      </c>
+      <c r="D14" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E14" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="F14" t="s" s="1">
         <v>66</v>
       </c>
-      <c r="B14" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="C14" t="s" s="1">
-        <v>12</v>
-      </c>
-      <c r="D14" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E14" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="F14" t="s" s="1">
+      <c r="G14" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="H14" t="s" s="1">
         <v>67</v>
       </c>
-      <c r="G14" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="H14" t="s" s="1">
+      <c r="I14" t="s" s="1">
         <v>68</v>
       </c>
-      <c r="I14" t="s" s="1">
-        <v>69</v>
-      </c>
       <c r="K14" t="s" s="1">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="1">
+        <v>69</v>
+      </c>
+      <c r="B15" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="C15" t="s" s="1">
+        <v>12</v>
+      </c>
+      <c r="D15" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E15" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="F15" t="s" s="1">
         <v>70</v>
       </c>
-      <c r="B15" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="C15" t="s" s="1">
-        <v>12</v>
-      </c>
-      <c r="D15" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E15" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="F15" t="s" s="1">
+      <c r="G15" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="H15" t="s" s="1">
         <v>71</v>
       </c>
-      <c r="G15" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="H15" t="s" s="1">
+      <c r="I15" t="s" s="1">
         <v>72</v>
       </c>
-      <c r="I15" t="s" s="1">
-        <v>73</v>
-      </c>
       <c r="K15" t="s" s="1">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="1">
+        <v>73</v>
+      </c>
+      <c r="B16" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="C16" t="s" s="1">
+        <v>12</v>
+      </c>
+      <c r="D16" t="s" s="1">
+        <v>60</v>
+      </c>
+      <c r="E16" t="s" s="1">
+        <v>61</v>
+      </c>
+      <c r="F16" t="s" s="1">
         <v>74</v>
       </c>
-      <c r="B16" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="C16" t="s" s="1">
-        <v>12</v>
-      </c>
-      <c r="D16" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E16" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="F16" t="s" s="1">
+      <c r="G16" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="H16" t="s" s="1">
         <v>75</v>
       </c>
-      <c r="G16" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="H16" t="s" s="1">
+      <c r="I16" t="s" s="1">
         <v>76</v>
       </c>
-      <c r="I16" t="s" s="1">
+      <c r="K16" t="s" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="s" s="1">
         <v>77</v>
       </c>
-      <c r="K16" t="s" s="1">
-        <v>27</v>
+      <c r="B17" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="C17" t="s" s="1">
+        <v>12</v>
+      </c>
+      <c r="D17" t="s" s="1">
+        <v>60</v>
+      </c>
+      <c r="E17" t="s" s="1">
+        <v>61</v>
+      </c>
+      <c r="F17" t="s" s="1">
+        <v>78</v>
+      </c>
+      <c r="G17" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="H17" t="s" s="1">
+        <v>79</v>
+      </c>
+      <c r="I17" t="s" s="1">
+        <v>80</v>
+      </c>
+      <c r="K17" t="s" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="s" s="1">
+        <v>81</v>
+      </c>
+      <c r="B18" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="C18" t="s" s="1">
+        <v>12</v>
+      </c>
+      <c r="D18" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E18" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="F18" t="s" s="1">
+        <v>82</v>
+      </c>
+      <c r="G18" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="H18" t="s" s="1">
+        <v>83</v>
+      </c>
+      <c r="I18" t="s" s="1">
+        <v>84</v>
+      </c>
+      <c r="K18" t="s" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="s" s="1">
+        <v>85</v>
+      </c>
+      <c r="B19" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="C19" t="s" s="1">
+        <v>12</v>
+      </c>
+      <c r="D19" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E19" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="F19" t="s" s="1">
+        <v>86</v>
+      </c>
+      <c r="G19" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="H19" t="s" s="1">
+        <v>87</v>
+      </c>
+      <c r="I19" t="s" s="1">
+        <v>88</v>
+      </c>
+      <c r="K19" t="s" s="1">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="s" s="1">
+        <v>89</v>
+      </c>
+      <c r="B20" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="C20" t="s" s="1">
+        <v>12</v>
+      </c>
+      <c r="D20" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="E20" t="s" s="1">
+        <v>13</v>
+      </c>
+      <c r="F20" t="s" s="1">
+        <v>90</v>
+      </c>
+      <c r="G20" t="s" s="1">
+        <v>15</v>
+      </c>
+      <c r="H20" t="s" s="1">
+        <v>91</v>
+      </c>
+      <c r="I20" t="s" s="1">
+        <v>92</v>
+      </c>
+      <c r="K20" t="s" s="1">
+        <v>30</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Keep single Excel export filename and improve pending update alerts
</commit_message>
<xml_diff>
--- a/downloads/Notificaciones Electrónicas.xlsx
+++ b/downloads/Notificaciones Electrónicas.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="200" uniqueCount="93">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="220" uniqueCount="100">
   <si>
     <t>Nro. Notificación</t>
   </si>
@@ -44,33 +44,63 @@
     <t>Estado de lectura</t>
   </si>
   <si>
+    <t>202600059037-1</t>
+  </si>
+  <si>
+    <t>RUC 20103117560</t>
+  </si>
+  <si>
+    <t>EMP REG DE SERV PUB DE ELECT DL NORTE SA</t>
+  </si>
+  <si>
+    <t>9994</t>
+  </si>
+  <si>
+    <t>TRANSPORTE FARO E.I.R.LTDA.</t>
+  </si>
+  <si>
+    <t>202600059037</t>
+  </si>
+  <si>
+    <t>Trámite Electrónico</t>
+  </si>
+  <si>
+    <t>APELACION DE CIEZA CAMPOS, ALDONIA, CONTRA EMP REG DE SERV PUB DE ELECT DEL NORTE SA RESOLUCION 25100096755 - REC R98510-A-2025 &amp;ndash; SUM. 40113401</t>
+  </si>
+  <si>
+    <t>16/03/2026 03:20:45 PM</t>
+  </si>
+  <si>
+    <t>Leída</t>
+  </si>
+  <si>
+    <t>202600058984-1</t>
+  </si>
+  <si>
+    <t>202600058984</t>
+  </si>
+  <si>
+    <t>APELACION DE LLONTOP YPARRAGUIRRE YVONNE CAROLINA CONTRA EMP REG DE SERV PUB DE ELECT DL NORTE SA RES1RAINST 25100097737 REC R99812-S-2026 SUM 36811768</t>
+  </si>
+  <si>
+    <t>16/03/2026 02:49:40 PM</t>
+  </si>
+  <si>
     <t>202600040663-4</t>
   </si>
   <si>
-    <t>RUC 20103117560</t>
-  </si>
-  <si>
-    <t>EMP REG DE SERV PUB DE ELECT DL NORTE SA</t>
-  </si>
-  <si>
     <t/>
   </si>
   <si>
     <t>202600040663</t>
   </si>
   <si>
-    <t>Trámite Electrónico</t>
-  </si>
-  <si>
     <t>Declarar la aplicación del silencio administrativo positivo.</t>
   </si>
   <si>
     <t>16/03/2026 02:00:59 PM</t>
   </si>
   <si>
-    <t>No leída</t>
-  </si>
-  <si>
     <t>202600039598-4</t>
   </si>
   <si>
@@ -104,9 +134,6 @@
     <t>16/03/2026 01:32:13 PM</t>
   </si>
   <si>
-    <t>Leída</t>
-  </si>
-  <si>
     <t>202500114631-4</t>
   </si>
   <si>
@@ -192,12 +219,6 @@
   </si>
   <si>
     <t>202600058734-1</t>
-  </si>
-  <si>
-    <t>9994</t>
-  </si>
-  <si>
-    <t>TRANSPORTE FARO E.I.R.LTDA.</t>
   </si>
   <si>
     <t>202600058734</t>
@@ -389,27 +410,27 @@
         <v>13</v>
       </c>
       <c r="E2" t="s" s="1">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F2" t="s" s="1">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G2" t="s" s="1">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H2" t="s" s="1">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="I2" t="s" s="1">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="K2" t="s" s="1">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s" s="1">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B3" t="s" s="1">
         <v>11</v>
@@ -421,27 +442,27 @@
         <v>13</v>
       </c>
       <c r="E3" t="s" s="1">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F3" t="s" s="1">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G3" t="s" s="1">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H3" t="s" s="1">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="I3" t="s" s="1">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="K3" t="s" s="1">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s" s="1">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B4" t="s" s="1">
         <v>11</v>
@@ -450,30 +471,30 @@
         <v>12</v>
       </c>
       <c r="D4" t="s" s="1">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="E4" t="s" s="1">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F4" t="s" s="1">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G4" t="s" s="1">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H4" t="s" s="1">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="I4" t="s" s="1">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="K4" t="s" s="1">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s" s="1">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B5" t="s" s="1">
         <v>11</v>
@@ -482,30 +503,30 @@
         <v>12</v>
       </c>
       <c r="D5" t="s" s="1">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="E5" t="s" s="1">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F5" t="s" s="1">
+        <v>30</v>
+      </c>
+      <c r="G5" t="s" s="1">
+        <v>16</v>
+      </c>
+      <c r="H5" t="s" s="1">
         <v>27</v>
       </c>
-      <c r="G5" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="H5" t="s" s="1">
-        <v>28</v>
-      </c>
       <c r="I5" t="s" s="1">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="K5" t="s" s="1">
-        <v>30</v>
+        <v>19</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s" s="1">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B6" t="s" s="1">
         <v>11</v>
@@ -514,30 +535,30 @@
         <v>12</v>
       </c>
       <c r="D6" t="s" s="1">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="E6" t="s" s="1">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F6" t="s" s="1">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="G6" t="s" s="1">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H6" t="s" s="1">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="I6" t="s" s="1">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="K6" t="s" s="1">
-        <v>30</v>
+        <v>19</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s" s="1">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B7" t="s" s="1">
         <v>11</v>
@@ -546,30 +567,30 @@
         <v>12</v>
       </c>
       <c r="D7" t="s" s="1">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="E7" t="s" s="1">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F7" t="s" s="1">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="G7" t="s" s="1">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H7" t="s" s="1">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="I7" t="s" s="1">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="K7" t="s" s="1">
-        <v>30</v>
+        <v>19</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s" s="1">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B8" t="s" s="1">
         <v>11</v>
@@ -578,30 +599,30 @@
         <v>12</v>
       </c>
       <c r="D8" t="s" s="1">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="E8" t="s" s="1">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F8" t="s" s="1">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="G8" t="s" s="1">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H8" t="s" s="1">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="I8" t="s" s="1">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="K8" t="s" s="1">
-        <v>30</v>
+        <v>19</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s" s="1">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="B9" t="s" s="1">
         <v>11</v>
@@ -610,30 +631,30 @@
         <v>12</v>
       </c>
       <c r="D9" t="s" s="1">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="E9" t="s" s="1">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F9" t="s" s="1">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G9" t="s" s="1">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H9" t="s" s="1">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="I9" t="s" s="1">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="K9" t="s" s="1">
-        <v>30</v>
+        <v>19</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s" s="1">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B10" t="s" s="1">
         <v>11</v>
@@ -642,30 +663,30 @@
         <v>12</v>
       </c>
       <c r="D10" t="s" s="1">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="E10" t="s" s="1">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F10" t="s" s="1">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G10" t="s" s="1">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H10" t="s" s="1">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="I10" t="s" s="1">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="K10" t="s" s="1">
-        <v>30</v>
+        <v>19</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s" s="1">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B11" t="s" s="1">
         <v>11</v>
@@ -674,30 +695,30 @@
         <v>12</v>
       </c>
       <c r="D11" t="s" s="1">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="E11" t="s" s="1">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F11" t="s" s="1">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="G11" t="s" s="1">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H11" t="s" s="1">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="I11" t="s" s="1">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="K11" t="s" s="1">
-        <v>30</v>
+        <v>19</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s" s="1">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="B12" t="s" s="1">
         <v>11</v>
@@ -706,30 +727,30 @@
         <v>12</v>
       </c>
       <c r="D12" t="s" s="1">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="E12" t="s" s="1">
-        <v>13</v>
+        <v>25</v>
       </c>
       <c r="F12" t="s" s="1">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G12" t="s" s="1">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H12" t="s" s="1">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="I12" t="s" s="1">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="K12" t="s" s="1">
-        <v>30</v>
+        <v>19</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s" s="1">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B13" t="s" s="1">
         <v>11</v>
@@ -738,62 +759,62 @@
         <v>12</v>
       </c>
       <c r="D13" t="s" s="1">
-        <v>60</v>
+        <v>25</v>
       </c>
       <c r="E13" t="s" s="1">
+        <v>25</v>
+      </c>
+      <c r="F13" t="s" s="1">
         <v>61</v>
       </c>
-      <c r="F13" t="s" s="1">
+      <c r="G13" t="s" s="1">
+        <v>16</v>
+      </c>
+      <c r="H13" t="s" s="1">
         <v>62</v>
       </c>
-      <c r="G13" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="H13" t="s" s="1">
+      <c r="I13" t="s" s="1">
         <v>63</v>
       </c>
-      <c r="I13" t="s" s="1">
-        <v>64</v>
-      </c>
       <c r="K13" t="s" s="1">
-        <v>30</v>
+        <v>19</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s" s="1">
+        <v>64</v>
+      </c>
+      <c r="B14" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="C14" t="s" s="1">
+        <v>12</v>
+      </c>
+      <c r="D14" t="s" s="1">
+        <v>25</v>
+      </c>
+      <c r="E14" t="s" s="1">
+        <v>25</v>
+      </c>
+      <c r="F14" t="s" s="1">
         <v>65</v>
       </c>
-      <c r="B14" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="C14" t="s" s="1">
-        <v>12</v>
-      </c>
-      <c r="D14" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E14" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="F14" t="s" s="1">
+      <c r="G14" t="s" s="1">
+        <v>16</v>
+      </c>
+      <c r="H14" t="s" s="1">
         <v>66</v>
       </c>
-      <c r="G14" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="H14" t="s" s="1">
+      <c r="I14" t="s" s="1">
         <v>67</v>
       </c>
-      <c r="I14" t="s" s="1">
-        <v>68</v>
-      </c>
       <c r="K14" t="s" s="1">
-        <v>30</v>
+        <v>19</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s" s="1">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B15" t="s" s="1">
         <v>11</v>
@@ -805,91 +826,91 @@
         <v>13</v>
       </c>
       <c r="E15" t="s" s="1">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F15" t="s" s="1">
+        <v>69</v>
+      </c>
+      <c r="G15" t="s" s="1">
+        <v>16</v>
+      </c>
+      <c r="H15" t="s" s="1">
         <v>70</v>
       </c>
-      <c r="G15" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="H15" t="s" s="1">
+      <c r="I15" t="s" s="1">
         <v>71</v>
       </c>
-      <c r="I15" t="s" s="1">
-        <v>72</v>
-      </c>
       <c r="K15" t="s" s="1">
-        <v>30</v>
+        <v>19</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s" s="1">
+        <v>72</v>
+      </c>
+      <c r="B16" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="C16" t="s" s="1">
+        <v>12</v>
+      </c>
+      <c r="D16" t="s" s="1">
+        <v>25</v>
+      </c>
+      <c r="E16" t="s" s="1">
+        <v>25</v>
+      </c>
+      <c r="F16" t="s" s="1">
         <v>73</v>
       </c>
-      <c r="B16" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="C16" t="s" s="1">
-        <v>12</v>
-      </c>
-      <c r="D16" t="s" s="1">
-        <v>60</v>
-      </c>
-      <c r="E16" t="s" s="1">
-        <v>61</v>
-      </c>
-      <c r="F16" t="s" s="1">
+      <c r="G16" t="s" s="1">
+        <v>16</v>
+      </c>
+      <c r="H16" t="s" s="1">
         <v>74</v>
       </c>
-      <c r="G16" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="H16" t="s" s="1">
+      <c r="I16" t="s" s="1">
         <v>75</v>
       </c>
-      <c r="I16" t="s" s="1">
-        <v>76</v>
-      </c>
       <c r="K16" t="s" s="1">
-        <v>30</v>
+        <v>19</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s" s="1">
+        <v>76</v>
+      </c>
+      <c r="B17" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="C17" t="s" s="1">
+        <v>12</v>
+      </c>
+      <c r="D17" t="s" s="1">
+        <v>25</v>
+      </c>
+      <c r="E17" t="s" s="1">
+        <v>25</v>
+      </c>
+      <c r="F17" t="s" s="1">
         <v>77</v>
       </c>
-      <c r="B17" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="C17" t="s" s="1">
-        <v>12</v>
-      </c>
-      <c r="D17" t="s" s="1">
-        <v>60</v>
-      </c>
-      <c r="E17" t="s" s="1">
-        <v>61</v>
-      </c>
-      <c r="F17" t="s" s="1">
+      <c r="G17" t="s" s="1">
+        <v>16</v>
+      </c>
+      <c r="H17" t="s" s="1">
         <v>78</v>
       </c>
-      <c r="G17" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="H17" t="s" s="1">
+      <c r="I17" t="s" s="1">
         <v>79</v>
       </c>
-      <c r="I17" t="s" s="1">
-        <v>80</v>
-      </c>
       <c r="K17" t="s" s="1">
-        <v>30</v>
+        <v>19</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s" s="1">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B18" t="s" s="1">
         <v>11</v>
@@ -901,27 +922,27 @@
         <v>13</v>
       </c>
       <c r="E18" t="s" s="1">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F18" t="s" s="1">
+        <v>81</v>
+      </c>
+      <c r="G18" t="s" s="1">
+        <v>16</v>
+      </c>
+      <c r="H18" t="s" s="1">
         <v>82</v>
       </c>
-      <c r="G18" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="H18" t="s" s="1">
+      <c r="I18" t="s" s="1">
         <v>83</v>
       </c>
-      <c r="I18" t="s" s="1">
-        <v>84</v>
-      </c>
       <c r="K18" t="s" s="1">
-        <v>30</v>
+        <v>19</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s" s="1">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="B19" t="s" s="1">
         <v>11</v>
@@ -933,54 +954,118 @@
         <v>13</v>
       </c>
       <c r="E19" t="s" s="1">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F19" t="s" s="1">
+        <v>85</v>
+      </c>
+      <c r="G19" t="s" s="1">
+        <v>16</v>
+      </c>
+      <c r="H19" t="s" s="1">
         <v>86</v>
       </c>
-      <c r="G19" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="H19" t="s" s="1">
+      <c r="I19" t="s" s="1">
         <v>87</v>
       </c>
-      <c r="I19" t="s" s="1">
-        <v>88</v>
-      </c>
       <c r="K19" t="s" s="1">
-        <v>30</v>
+        <v>19</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s" s="1">
+        <v>88</v>
+      </c>
+      <c r="B20" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="C20" t="s" s="1">
+        <v>12</v>
+      </c>
+      <c r="D20" t="s" s="1">
+        <v>25</v>
+      </c>
+      <c r="E20" t="s" s="1">
+        <v>25</v>
+      </c>
+      <c r="F20" t="s" s="1">
         <v>89</v>
       </c>
-      <c r="B20" t="s" s="1">
-        <v>11</v>
-      </c>
-      <c r="C20" t="s" s="1">
-        <v>12</v>
-      </c>
-      <c r="D20" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="E20" t="s" s="1">
-        <v>13</v>
-      </c>
-      <c r="F20" t="s" s="1">
+      <c r="G20" t="s" s="1">
+        <v>16</v>
+      </c>
+      <c r="H20" t="s" s="1">
         <v>90</v>
       </c>
-      <c r="G20" t="s" s="1">
-        <v>15</v>
-      </c>
-      <c r="H20" t="s" s="1">
+      <c r="I20" t="s" s="1">
         <v>91</v>
       </c>
-      <c r="I20" t="s" s="1">
+      <c r="K20" t="s" s="1">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="s" s="1">
         <v>92</v>
       </c>
-      <c r="K20" t="s" s="1">
-        <v>30</v>
+      <c r="B21" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="C21" t="s" s="1">
+        <v>12</v>
+      </c>
+      <c r="D21" t="s" s="1">
+        <v>25</v>
+      </c>
+      <c r="E21" t="s" s="1">
+        <v>25</v>
+      </c>
+      <c r="F21" t="s" s="1">
+        <v>93</v>
+      </c>
+      <c r="G21" t="s" s="1">
+        <v>16</v>
+      </c>
+      <c r="H21" t="s" s="1">
+        <v>94</v>
+      </c>
+      <c r="I21" t="s" s="1">
+        <v>95</v>
+      </c>
+      <c r="K21" t="s" s="1">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s" s="1">
+        <v>96</v>
+      </c>
+      <c r="B22" t="s" s="1">
+        <v>11</v>
+      </c>
+      <c r="C22" t="s" s="1">
+        <v>12</v>
+      </c>
+      <c r="D22" t="s" s="1">
+        <v>25</v>
+      </c>
+      <c r="E22" t="s" s="1">
+        <v>25</v>
+      </c>
+      <c r="F22" t="s" s="1">
+        <v>97</v>
+      </c>
+      <c r="G22" t="s" s="1">
+        <v>16</v>
+      </c>
+      <c r="H22" t="s" s="1">
+        <v>98</v>
+      </c>
+      <c r="I22" t="s" s="1">
+        <v>99</v>
+      </c>
+      <c r="K22" t="s" s="1">
+        <v>19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>